<commit_message>
Added the pipeline for boats
</commit_message>
<xml_diff>
--- a/infrastructure/config/ToScrape.xlsx
+++ b/infrastructure/config/ToScrape.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\beepe\Desktop\Yacht\infrastructure\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB0E1AC4-F259-45F8-82C9-97061B295E71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{873CA29A-0776-4BBD-8F89-9FFEFE56B606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Glosary" sheetId="3" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
   <si>
     <t>Regatta Name</t>
   </si>
@@ -45,13 +45,16 @@
   </si>
   <si>
     <t>PDF Route</t>
+  </si>
+  <si>
+    <t>Year</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -63,6 +66,14 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -104,12 +115,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -400,37 +412,41 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="117" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.36328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="117" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C2" s="1"/>
+    <row r="2" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="D2" s="1"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="C3" s="2"/>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D3" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -439,26 +455,30 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{749A66F4-3D21-43CF-A710-31B74BD3E465}">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="12.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="83.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.453125" customWidth="1"/>
+    <col min="3" max="3" width="11.7265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="83.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" s="3" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Refactoring codes after checking the boats pipeline
</commit_message>
<xml_diff>
--- a/infrastructure/config/ToScrape.xlsx
+++ b/infrastructure/config/ToScrape.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\beepe\Desktop\Yacht\infrastructure\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{873CA29A-0776-4BBD-8F89-9FFEFE56B606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D329B43-280C-4834-BB69-A713AA476DAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="11">
   <si>
     <t>Regatta Name</t>
   </si>
@@ -48,6 +48,18 @@
   </si>
   <si>
     <t>Year</t>
+  </si>
+  <si>
+    <t>6 Metre British Open Nationals</t>
+  </si>
+  <si>
+    <t>https://yachtscoring.com/event_results_cumulative/16953</t>
+  </si>
+  <si>
+    <t>yachtscoring</t>
+  </si>
+  <si>
+    <t>6 metre</t>
   </si>
 </sst>
 </file>
@@ -87,7 +99,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -95,31 +107,13 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="FFCCCCCC"/>
-      </left>
-      <right style="medium">
-        <color rgb="FFCCCCCC"/>
-      </right>
-      <top style="medium">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FFCCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -416,39 +410,59 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4.6328125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4.81640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="10.36328125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="117" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="D2" s="1"/>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2">
+        <v>2025</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="D3" s="2"/>
+      <c r="D3" s="1"/>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D2" r:id="rId1" xr:uid="{8B3C24CD-0C18-4C0E-814D-248E50F099DF}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -466,19 +480,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Added to save raw values into prenormalization
</commit_message>
<xml_diff>
--- a/infrastructure/config/ToScrape.xlsx
+++ b/infrastructure/config/ToScrape.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\beepe\Desktop\Yacht\infrastructure\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{068C60B7-BBD7-4A52-A93B-74F52DAF4F64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD97067-B4B4-43D2-9B0C-3083EDF3767E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="193">
   <si>
     <t>Regatta Name</t>
   </si>
@@ -1028,8 +1028,8 @@
     <col min="2" max="2" width="5.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="97.36328125" customWidth="1"/>
-    <col min="6" max="6" width="13" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -2538,7 +2538,10 @@
         <v>191</v>
       </c>
       <c r="E71" s="11">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G71" s="11" t="s">
+        <v>158</v>
       </c>
     </row>
     <row r="72" spans="1:7">
@@ -2555,7 +2558,10 @@
         <v>192</v>
       </c>
       <c r="E72" s="11">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="G72" s="11" t="s">
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes in scraper sailwave_pdf
</commit_message>
<xml_diff>
--- a/infrastructure/config/ToScrape.xlsx
+++ b/infrastructure/config/ToScrape.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\beepe\Desktop\Yacht\infrastructure\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AD97067-B4B4-43D2-9B0C-3083EDF3767E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09EF763-79E4-4760-8F8B-8DA8577C7C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Glosary" sheetId="3" r:id="rId1"/>
@@ -1021,7 +1021,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G72"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="39" bestFit="1" customWidth="1"/>
@@ -2563,6 +2563,9 @@
       <c r="G72" s="11" t="s">
         <v>158</v>
       </c>
+    </row>
+    <row r="73" spans="1:7">
+      <c r="A73" s="3"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G69" xr:uid="{00000000-0001-0000-0000-000000000000}">
@@ -2783,7 +2786,7 @@
         <v>0</v>
       </c>
       <c r="G9" t="s">
-        <v>187</v>
+        <v>158</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes in boats pipelines
</commit_message>
<xml_diff>
--- a/infrastructure/config/ToScrape.xlsx
+++ b/infrastructure/config/ToScrape.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\beepe\Desktop\Yacht\infrastructure\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A09EF763-79E4-4760-8F8B-8DA8577C7C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E41CADF5-E28A-4955-8CB2-189610806A75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Glosary" sheetId="3" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="345" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="194">
   <si>
     <t>Regatta Name</t>
   </si>
@@ -92,9 +92,6 @@
     <t>RORC Easter Regatta</t>
   </si>
   <si>
-    <t>Vice Admiral’s Cup</t>
-  </si>
-  <si>
     <t>Poole Regatta</t>
   </si>
   <si>
@@ -140,15 +137,6 @@
     <t>5.5 Metre UK Nationals</t>
   </si>
   <si>
-    <t>Sigma 33 National Champ.</t>
-  </si>
-  <si>
-    <t>Sonata National Champ.</t>
-  </si>
-  <si>
-    <t>Flying 15 National Champ.</t>
-  </si>
-  <si>
     <t>Contessa 32 Nationals</t>
   </si>
   <si>
@@ -609,6 +597,21 @@
   </si>
   <si>
     <t>https://www.ryyc.org.uk/series/11655</t>
+  </si>
+  <si>
+    <t>Sonata National Championship</t>
+  </si>
+  <si>
+    <t>Sigma 33 National Championship</t>
+  </si>
+  <si>
+    <t>Flying 15 National Championship</t>
+  </si>
+  <si>
+    <t>Flying 15</t>
+  </si>
+  <si>
+    <t>Vice Admiral's Cup</t>
   </si>
 </sst>
 </file>
@@ -1052,49 +1055,49 @@
         <v>4</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="B2" s="6">
         <v>2025</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="E2" s="6">
         <v>0</v>
       </c>
       <c r="F2" s="6"/>
       <c r="G2" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:7">
       <c r="A3" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B3" s="6">
         <v>2025</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="E3" s="6">
         <v>0</v>
       </c>
       <c r="F3" s="6"/>
       <c r="G3" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:7">
@@ -1114,221 +1117,221 @@
         <v>0</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="5" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="B5" s="6">
         <v>2025</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="E5" s="6">
         <v>0</v>
       </c>
       <c r="F5" s="6"/>
       <c r="G5" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B6" s="6">
         <v>2025</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D6" s="14" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="E6" s="6">
         <v>0</v>
       </c>
       <c r="F6" s="6"/>
       <c r="G6" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B7" s="6">
         <v>2025</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="E7" s="6">
         <v>0</v>
       </c>
       <c r="F7" s="6"/>
       <c r="G7" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B8" s="6">
         <v>2025</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="E8" s="6">
         <v>0</v>
       </c>
       <c r="F8" s="6"/>
       <c r="G8" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="10" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" s="6">
+        <v>2025</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D9" s="6" t="s">
         <v>160</v>
-      </c>
-      <c r="B9" s="6">
-        <v>2025</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>164</v>
       </c>
       <c r="E9" s="6">
         <v>0</v>
       </c>
       <c r="F9" s="6"/>
       <c r="G9" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B10" s="6">
         <v>2025</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="E10" s="6">
         <v>0</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="10" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
       <c r="B11" s="6">
         <v>2025</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="E11" s="6">
         <v>0</v>
       </c>
       <c r="F11" s="6"/>
       <c r="G11" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="12" spans="1:7">
       <c r="A12" s="5" t="s">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="B12" s="6">
         <v>2025</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="E12" s="6">
         <v>0</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" spans="1:7">
       <c r="A13" s="12" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B13" s="11">
         <v>2025</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="E13" s="6">
         <v>0</v>
       </c>
       <c r="G13" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="14" spans="1:7">
       <c r="A14" s="5" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14" s="6">
         <v>2025</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>98</v>
+        <v>94</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="E14" s="6">
         <v>0</v>
       </c>
       <c r="F14" s="6"/>
       <c r="G14" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1339,187 +1342,189 @@
         <v>2025</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E15" s="6">
         <v>0</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="16" spans="1:7">
       <c r="A16" s="5" t="s">
-        <v>38</v>
+        <v>191</v>
       </c>
       <c r="B16" s="6">
         <v>2025</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="E16" s="6">
         <v>0</v>
       </c>
-      <c r="F16" s="6"/>
+      <c r="F16" s="6" t="s">
+        <v>192</v>
+      </c>
       <c r="G16" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="17" spans="1:7">
       <c r="A17" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B17" s="6">
         <v>2025</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="E17" s="6">
         <v>0</v>
       </c>
       <c r="F17" s="6"/>
       <c r="G17" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="18" spans="1:7">
       <c r="A18" s="5" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B18" s="6">
         <v>2025</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E18" s="6">
         <v>0</v>
       </c>
       <c r="F18" s="6"/>
       <c r="G18" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="19" spans="1:7">
       <c r="A19" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B19" s="6">
         <v>2025</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="E19" s="6">
         <v>0</v>
       </c>
       <c r="F19" s="6"/>
       <c r="G19" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="20" spans="1:7">
       <c r="A20" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B20" s="6">
         <v>2025</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="E20" s="6">
         <v>0</v>
       </c>
       <c r="F20" s="6"/>
       <c r="G20" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="21" spans="1:7">
       <c r="A21" s="5" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B21" s="6">
         <v>2025</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="E21" s="6">
         <v>0</v>
       </c>
       <c r="F21" s="6"/>
       <c r="G21" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22" spans="1:7">
       <c r="A22" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B22" s="6">
         <v>2025</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="E22" s="6">
         <v>0</v>
       </c>
       <c r="F22" s="6"/>
       <c r="G22" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="23" spans="1:7">
       <c r="A23" s="9" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="B23" s="6">
         <v>2025</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D23" s="6" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="E23" s="6">
         <v>0</v>
       </c>
       <c r="F23" s="6"/>
       <c r="G23" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="24" spans="1:7">
@@ -1530,38 +1535,38 @@
         <v>2025</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E24" s="6">
         <v>0</v>
       </c>
       <c r="F24" s="6"/>
       <c r="G24" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="25" spans="1:7">
       <c r="A25" s="5" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B25" s="6">
         <v>2025</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="E25" s="6">
         <v>0</v>
       </c>
       <c r="F25" s="6"/>
       <c r="G25" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="26" spans="1:7">
@@ -1575,16 +1580,16 @@
         <v>9</v>
       </c>
       <c r="D26" s="6" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E26" s="6">
         <v>0</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="27" spans="1:7">
@@ -1595,143 +1600,143 @@
         <v>2025</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D27" s="6" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="E27" s="6">
         <v>0</v>
       </c>
       <c r="F27" s="6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="28" spans="1:7">
       <c r="A28" s="5" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B28" s="6">
         <v>2025</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D28" s="6" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="E28" s="6">
         <v>0</v>
       </c>
       <c r="F28" s="6"/>
       <c r="G28" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="29" spans="1:7">
       <c r="A29" s="13" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B29" s="11">
         <v>2025</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="E29" s="6">
         <v>0</v>
       </c>
       <c r="G29" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="30" spans="1:7">
       <c r="A30" s="5" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B30" s="6">
         <v>2025</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D30" s="14" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="E30" s="6">
         <v>0</v>
       </c>
       <c r="F30" s="6"/>
       <c r="G30" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="31" spans="1:7">
       <c r="A31" s="9" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="B31" s="6">
         <v>2025</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="E31" s="6">
         <v>0</v>
       </c>
       <c r="F31" s="6"/>
       <c r="G31" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="32" spans="1:7">
       <c r="A32" s="13" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B32" s="11">
         <v>2025</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="E32" s="6">
         <v>0</v>
       </c>
       <c r="G32" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="33" spans="1:7">
       <c r="A33" s="5" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="B33" s="6">
         <v>2025</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D33" s="6" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="E33" s="6">
         <v>0</v>
       </c>
       <c r="F33" s="6"/>
       <c r="G33" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="34" spans="1:7">
@@ -1742,59 +1747,59 @@
         <v>2025</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="D34" s="6" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="E34" s="6">
         <v>0</v>
       </c>
       <c r="F34" s="6"/>
       <c r="G34" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="35" spans="1:7">
       <c r="A35" s="5" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="B35" s="6">
         <v>2025</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D35" s="6" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="E35" s="6">
         <v>0</v>
       </c>
       <c r="F35" s="6"/>
       <c r="G35" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="36" spans="1:7">
       <c r="A36" s="5" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="B36" s="6">
         <v>2025</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D36" s="6" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E36" s="6">
         <v>0</v>
       </c>
       <c r="F36" s="6"/>
       <c r="G36" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="37" spans="1:7">
@@ -1805,145 +1810,145 @@
         <v>2025</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D37" s="6" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
       <c r="E37" s="6">
         <v>0</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="38" spans="1:7">
       <c r="A38" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B38" s="6">
         <v>2025</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D38" s="6" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E38" s="6">
         <v>0</v>
       </c>
       <c r="F38" s="6"/>
       <c r="G38" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="39" spans="1:7">
       <c r="A39" s="5" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B39" s="6">
         <v>2025</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D39" s="6" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="E39" s="6">
         <v>0</v>
       </c>
       <c r="F39" s="6"/>
       <c r="G39" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="40" spans="1:7">
       <c r="A40" s="9" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="B40" s="6">
         <v>2025</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D40" s="6" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="E40" s="6">
         <v>0</v>
       </c>
       <c r="F40" s="6"/>
       <c r="G40" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="41" spans="1:7">
       <c r="A41" s="5" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="B41" s="6">
         <v>2025</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D41" s="6" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="E41" s="6">
         <v>0</v>
       </c>
       <c r="F41" s="6"/>
       <c r="G41" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="42" spans="1:7">
       <c r="A42" s="5" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="B42" s="6">
         <v>2025</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D42" s="6" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="E42" s="6">
         <v>0</v>
       </c>
       <c r="F42" s="6"/>
       <c r="G42" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="43" spans="1:7">
       <c r="A43" s="5" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="B43" s="6">
         <v>2025</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D43" s="6" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="E43" s="6">
         <v>0</v>
       </c>
       <c r="F43" s="6"/>
       <c r="G43" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="44" spans="1:7">
@@ -1957,161 +1962,161 @@
         <v>9</v>
       </c>
       <c r="D44" s="14" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="E44" s="6">
         <v>0</v>
       </c>
       <c r="F44" s="6"/>
       <c r="G44" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="45" spans="1:7">
       <c r="A45" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B45" s="6">
         <v>2025</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D45" s="6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E45" s="6">
         <v>0</v>
       </c>
       <c r="F45" s="6"/>
       <c r="G45" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="46" spans="1:7">
       <c r="A46" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B46" s="6">
         <v>2025</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D46" s="6" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="E46" s="6">
         <v>0</v>
       </c>
       <c r="F46" s="6"/>
       <c r="G46" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="47" spans="1:7">
       <c r="A47" s="9" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B47" s="6">
         <v>2024</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D47" s="6" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="E47" s="6">
         <v>0</v>
       </c>
       <c r="F47" s="6"/>
       <c r="G47" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="48" spans="1:7">
       <c r="A48" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B48" s="6">
         <v>2025</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D48" s="6" t="s">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E48" s="6">
         <v>0</v>
       </c>
       <c r="F48" s="6"/>
       <c r="G48" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="49" spans="1:7">
       <c r="A49" s="8" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="B49" s="6">
         <v>2025</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D49" s="6" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="E49" s="6">
         <v>0</v>
       </c>
       <c r="F49" s="6"/>
       <c r="G49" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="50" spans="1:7">
       <c r="A50" s="9" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B50" s="6">
         <v>2025</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D50" s="6" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="E50" s="6">
         <v>0</v>
       </c>
       <c r="F50" s="6"/>
       <c r="G50" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="51" spans="1:7">
       <c r="A51" s="5" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="B51" s="6">
         <v>2025</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D51" s="6" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="E51" s="6">
         <v>0</v>
       </c>
       <c r="F51" s="6"/>
       <c r="G51" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="52" spans="1:7">
@@ -2122,17 +2127,17 @@
         <v>2025</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D52" s="6" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="E52" s="6">
         <v>0</v>
       </c>
       <c r="F52" s="6"/>
       <c r="G52" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="53" spans="1:7">
@@ -2143,238 +2148,238 @@
         <v>2025</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D53" s="6" t="s">
-        <v>61</v>
+        <v>57</v>
       </c>
       <c r="E53" s="6">
         <v>0</v>
       </c>
       <c r="F53" s="6"/>
       <c r="G53" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="54" spans="1:7">
       <c r="A54" s="5" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B54" s="6">
         <v>2025</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D54" s="6" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E54" s="6">
         <v>0</v>
       </c>
       <c r="F54" s="6"/>
       <c r="G54" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="55" spans="1:7">
       <c r="A55" s="5" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B55" s="6">
         <v>2025</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D55" s="6" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="E55" s="6">
         <v>0</v>
       </c>
       <c r="F55" s="6" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="G55" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="56" spans="1:7">
       <c r="A56" s="5" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B56" s="6">
         <v>2025</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D56" s="6" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E56" s="6">
         <v>0</v>
       </c>
       <c r="F56" s="6"/>
       <c r="G56" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="57" spans="1:7">
       <c r="A57" s="5" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B57" s="6">
         <v>2025</v>
       </c>
       <c r="C57" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="D57" s="6" t="s">
         <v>75</v>
-      </c>
-      <c r="D57" s="6" t="s">
-        <v>79</v>
       </c>
       <c r="E57" s="6">
         <v>0</v>
       </c>
       <c r="F57" s="6"/>
       <c r="G57" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="58" spans="1:7">
       <c r="A58" s="12" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="B58" s="11">
         <v>2024</v>
       </c>
       <c r="C58" s="11" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="E58" s="6">
         <v>0</v>
       </c>
       <c r="G58" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="59" spans="1:7">
       <c r="A59" s="9" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B59" s="6">
         <v>2025</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D59" s="6" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="E59" s="6">
         <v>0</v>
       </c>
       <c r="F59" s="6"/>
       <c r="G59" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="60" spans="1:7">
       <c r="A60" s="5" t="s">
-        <v>36</v>
+        <v>190</v>
       </c>
       <c r="B60" s="6">
         <v>2025</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="D60" s="6" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E60" s="6">
         <v>0</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="61" spans="1:7">
       <c r="A61" s="13" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B61" s="11">
         <v>2025</v>
       </c>
       <c r="C61" s="11" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D61" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="E61" s="11">
         <v>0</v>
       </c>
       <c r="G61" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="62" spans="1:7">
       <c r="A62" s="5" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="B62" s="6">
         <v>2025</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D62" s="6" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E62" s="6">
         <v>0</v>
       </c>
       <c r="F62" s="6" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="63" spans="1:7">
       <c r="A63" s="5" t="s">
-        <v>37</v>
+        <v>189</v>
       </c>
       <c r="B63" s="6">
         <v>2025</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D63" s="14" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E63" s="6">
         <v>0</v>
       </c>
       <c r="F63" s="6" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="G63" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="64" spans="1:7">
       <c r="A64" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B64" s="6">
         <v>2025</v>
@@ -2383,42 +2388,42 @@
         <v>9</v>
       </c>
       <c r="D64" s="6" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="E64" s="6">
         <v>0</v>
       </c>
       <c r="F64" s="6" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="G64" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="65" spans="1:7">
       <c r="A65" s="5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B65" s="6">
         <v>2025</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="D65" s="6" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E65" s="6">
         <v>0</v>
       </c>
       <c r="F65" s="6"/>
       <c r="G65" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="66" spans="1:7">
       <c r="A66" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B66" s="6">
         <v>2025</v>
@@ -2427,37 +2432,37 @@
         <v>9</v>
       </c>
       <c r="D66" s="6" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="E66" s="6">
         <v>0</v>
       </c>
       <c r="F66" s="6" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="G66" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="67" spans="1:7">
-      <c r="A67" s="5" t="s">
-        <v>20</v>
+      <c r="A67" s="3" t="s">
+        <v>193</v>
       </c>
       <c r="B67" s="6">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D67" s="6" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="E67" s="6">
         <v>0</v>
       </c>
       <c r="F67" s="6"/>
       <c r="G67" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="68" spans="1:7">
@@ -2468,22 +2473,22 @@
         <v>2025</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D68" s="6" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E68" s="6">
         <v>0</v>
       </c>
       <c r="F68" s="6"/>
       <c r="G68" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="69" spans="1:7">
       <c r="A69" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B69" s="6">
         <v>2024</v>
@@ -2492,76 +2497,76 @@
         <v>9</v>
       </c>
       <c r="D69" s="6" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="E69" s="6">
         <v>0</v>
       </c>
       <c r="F69" s="6" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="G69" s="6" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="70" spans="1:7">
       <c r="A70" s="13" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B70" s="11">
         <v>2025</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D70" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="E70" s="11">
         <v>0</v>
       </c>
       <c r="G70" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="71" spans="1:7">
       <c r="A71" s="13" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B71" s="11">
         <v>2025</v>
       </c>
       <c r="C71" s="11" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D71" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="E71" s="11">
         <v>0</v>
       </c>
       <c r="G71" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="72" spans="1:7">
       <c r="A72" s="13" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B72" s="11">
         <v>2025</v>
       </c>
       <c r="C72" s="11" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="D72" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="E72" s="11">
         <v>0</v>
       </c>
       <c r="G72" s="11" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="73" spans="1:7">
@@ -2620,173 +2625,173 @@
         <v>4</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="15" thickBot="1">
       <c r="A2" s="2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="B2">
         <v>2025</v>
       </c>
       <c r="C2" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="E2">
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="15" thickBot="1">
       <c r="A3" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B3">
         <v>2025</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="D3" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="4" spans="1:7">
       <c r="A4" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B4">
         <v>2025</v>
       </c>
       <c r="C4" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D4" t="s">
+        <v>145</v>
+      </c>
+      <c r="E4">
+        <v>0</v>
+      </c>
+      <c r="F4" t="s">
         <v>149</v>
       </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4" t="s">
-        <v>153</v>
-      </c>
       <c r="G4" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B5">
         <v>2025</v>
       </c>
       <c r="C5" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D5" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="G5" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B6">
         <v>2025</v>
       </c>
       <c r="C6" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D6" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
       <c r="G6" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B7">
         <v>2025</v>
       </c>
       <c r="C7" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D7" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="E7">
         <v>0</v>
       </c>
       <c r="G7" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B8">
         <v>2025</v>
       </c>
       <c r="C8" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D8" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="E8">
         <v>0</v>
       </c>
       <c r="G8" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B9">
         <v>2025</v>
       </c>
       <c r="C9" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D9" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="E9">
         <v>0</v>
       </c>
       <c r="G9" t="s">
-        <v>158</v>
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added log to all scrapers
</commit_message>
<xml_diff>
--- a/infrastructure/config/ToScrape.xlsx
+++ b/infrastructure/config/ToScrape.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\beepe\Desktop\Yacht\infrastructure\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E41CADF5-E28A-4955-8CB2-189610806A75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6641F443-A983-4737-A144-2B90703A8556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="196">
   <si>
     <t>Regatta Name</t>
   </si>
@@ -612,6 +612,12 @@
   </si>
   <si>
     <t>Vice Admiral's Cup</t>
+  </si>
+  <si>
+    <t>https://sailracehq.com/results/event/7318e12f-d43e-47c2-9cbd-263d8e03d7b2/2026</t>
+  </si>
+  <si>
+    <t>Por scraear</t>
   </si>
 </sst>
 </file>
@@ -2570,7 +2576,24 @@
       </c>
     </row>
     <row r="73" spans="1:7">
-      <c r="A73" s="3"/>
+      <c r="A73" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="B73" s="11">
+        <v>2026</v>
+      </c>
+      <c r="C73" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="D73" t="s">
+        <v>194</v>
+      </c>
+      <c r="E73" s="11">
+        <v>1</v>
+      </c>
+      <c r="G73" s="11" t="s">
+        <v>195</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:G69" xr:uid="{00000000-0001-0000-0000-000000000000}">

</xml_diff>

<commit_message>
Added new scraper to manage2sail webpage
</commit_message>
<xml_diff>
--- a/infrastructure/config/ToScrape.xlsx
+++ b/infrastructure/config/ToScrape.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\beepe\Desktop\Yacht\infrastructure\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6641F443-A983-4737-A144-2B90703A8556}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ED84299-F3DF-4FE1-9FF4-C07036E2B78E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="201">
   <si>
     <t>Regatta Name</t>
   </si>
@@ -617,7 +617,22 @@
     <t>https://sailracehq.com/results/event/7318e12f-d43e-47c2-9cbd-263d8e03d7b2/2026</t>
   </si>
   <si>
-    <t>Por scraear</t>
+    <t>Southern Straits</t>
+  </si>
+  <si>
+    <t>clubspot</t>
+  </si>
+  <si>
+    <t>https://theclubspot.com/regatta/s0LES7S2b0/results</t>
+  </si>
+  <si>
+    <t>J70 Easter Regatta</t>
+  </si>
+  <si>
+    <t>manage2sail</t>
+  </si>
+  <si>
+    <t>https://manage2sail.com/en-US/event/f8f6e703-4f4a-40ac-a422-273f7e15b07e#!/results?classId=2b1d1991-f501-4c22-a417-45687cc0b1cb</t>
   </si>
 </sst>
 </file>
@@ -1030,7 +1045,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G73"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="39" bestFit="1" customWidth="1"/>
@@ -2589,10 +2604,53 @@
         <v>194</v>
       </c>
       <c r="E73" s="11">
+        <v>0</v>
+      </c>
+      <c r="G73" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7">
+      <c r="A74" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="B74" s="11">
+        <v>2026</v>
+      </c>
+      <c r="C74" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="D74" t="s">
+        <v>197</v>
+      </c>
+      <c r="E74" s="11">
+        <v>0</v>
+      </c>
+      <c r="G74" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7">
+      <c r="A75" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="B75" s="11">
+        <v>2026</v>
+      </c>
+      <c r="C75" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="D75" t="s">
+        <v>200</v>
+      </c>
+      <c r="E75" s="11">
         <v>1</v>
       </c>
-      <c r="G73" s="11" t="s">
-        <v>195</v>
+      <c r="F75" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G75" s="11" t="s">
+        <v>154</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new scraper 'Sailti' and new order in scraping folder
</commit_message>
<xml_diff>
--- a/infrastructure/config/ToScrape.xlsx
+++ b/infrastructure/config/ToScrape.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\beepe\Desktop\Yacht\infrastructure\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ED84299-F3DF-4FE1-9FF4-C07036E2B78E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6D793BB-08CD-4A07-88CA-BDF773BE8541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="204">
   <si>
     <t>Regatta Name</t>
   </si>
@@ -633,6 +633,15 @@
   </si>
   <si>
     <t>https://manage2sail.com/en-US/event/f8f6e703-4f4a-40ac-a422-273f7e15b07e#!/results?classId=2b1d1991-f501-4c22-a417-45687cc0b1cb</t>
+  </si>
+  <si>
+    <t>VI Trofeo Natalio Comas</t>
+  </si>
+  <si>
+    <t>https://www.federacionbalearvela.org/es/default/results/resultsall/return/results/text/campeonato-mallorca-vi-trofeo-natalio-comas-ilca-4-ilca-6-ilca-master</t>
+  </si>
+  <si>
+    <t>sailti</t>
   </si>
 </sst>
 </file>
@@ -1045,7 +1054,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="39" bestFit="1" customWidth="1"/>
@@ -2644,13 +2653,30 @@
         <v>200</v>
       </c>
       <c r="E75" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F75" s="11" t="s">
         <v>64</v>
       </c>
       <c r="G75" s="11" t="s">
         <v>154</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7">
+      <c r="A76" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="B76" s="11">
+        <v>2026</v>
+      </c>
+      <c r="C76" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="D76" t="s">
+        <v>202</v>
+      </c>
+      <c r="E76" s="11">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new scraper sportspafe
</commit_message>
<xml_diff>
--- a/infrastructure/config/ToScrape.xlsx
+++ b/infrastructure/config/ToScrape.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\beepe\Desktop\Yacht\infrastructure\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6D793BB-08CD-4A07-88CA-BDF773BE8541}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83CC663A-F665-4C5E-B6E3-98746494F572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Glosary" sheetId="3" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="209">
   <si>
     <t>Regatta Name</t>
   </si>
@@ -642,6 +642,21 @@
   </si>
   <si>
     <t>sailti</t>
+  </si>
+  <si>
+    <t>Australian International 2.4 Metre Class National Championship</t>
+  </si>
+  <si>
+    <t>sportspage</t>
+  </si>
+  <si>
+    <t>https://www.sportspage.com.au/yacht_clubs/rfbyc/Int2-4Nationals2026/International_2_4mR_WA_State_Championship.htm</t>
+  </si>
+  <si>
+    <t>https://www.sportspage.com.au/yacht_clubs/rfbyc/Int2-4Nationals2026/International_2_4mR_National_Championship.htm</t>
+  </si>
+  <si>
+    <t>2.4 Metre</t>
   </si>
 </sst>
 </file>
@@ -1054,13 +1069,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="39" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="51.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="5.26953125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.90625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="97.36328125" customWidth="1"/>
+    <col min="4" max="4" width="199.36328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="15.90625" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="16.90625" bestFit="1" customWidth="1"/>
   </cols>
@@ -2676,7 +2691,50 @@
         <v>202</v>
       </c>
       <c r="E76" s="11">
+        <v>0</v>
+      </c>
+      <c r="G76" s="11" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7">
+      <c r="A77" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B77" s="11">
+        <v>2026</v>
+      </c>
+      <c r="C77" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="D77" t="s">
+        <v>206</v>
+      </c>
+      <c r="E77" s="11">
         <v>1</v>
+      </c>
+      <c r="F77" s="11" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7">
+      <c r="A78" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="B78" s="11">
+        <v>2026</v>
+      </c>
+      <c r="C78" s="11" t="s">
+        <v>205</v>
+      </c>
+      <c r="D78" t="s">
+        <v>207</v>
+      </c>
+      <c r="E78" s="11">
+        <v>1</v>
+      </c>
+      <c r="F78" s="11" t="s">
+        <v>208</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes to creata a remote database
</commit_message>
<xml_diff>
--- a/infrastructure/config/ToScrape.xlsx
+++ b/infrastructure/config/ToScrape.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\beepe\Desktop\Yacht\infrastructure\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B45FD674-DBB2-4D40-A773-6EAAE1432B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47B4F3EC-F148-498F-BC59-947E783DA09D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2789,7 +2789,7 @@
         <v>212</v>
       </c>
       <c r="E80" s="11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F80" s="11" t="s">
         <v>69</v>

</xml_diff>

<commit_message>
Add club alias review and syn workflow
</commit_message>
<xml_diff>
--- a/infrastructure/config/ToScrape.xlsx
+++ b/infrastructure/config/ToScrape.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\beepe\Desktop\Yacht\infrastructure\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB169996-EF54-4B34-A61C-62023F761C5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90775AA6-CC9D-4C3A-8DB8-7D6FD018C8BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2342,7 +2342,7 @@
         <v>216</v>
       </c>
       <c r="E58" s="6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G58" s="6" t="s">
         <v>153</v>

</xml_diff>